<commit_message>
fix: update negative test highlights mismatch
</commit_message>
<xml_diff>
--- a/rules/CORE-000016/negative/03/data/unit-test-coreid-CG0089-negative.xlsx
+++ b/rules/CORE-000016/negative/03/data/unit-test-coreid-CG0089-negative.xlsx
@@ -2898,7 +2898,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Not in dataset</t>
+          <t>[ABSENT]</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Not in dataset</t>
+          <t>[ABSENT]</t>
         </is>
       </c>
     </row>
@@ -3010,7 +3010,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Not in dataset</t>
+          <t>[ABSENT]</t>
         </is>
       </c>
     </row>

</xml_diff>